<commit_message>
Load records for pivot tables into XLPivotTableCache. Doesn't write them out yet.
The modified test fiels contained values for a shared items in a table the definition shouldn't contains (e.g. pure numeric values not found in original table definition).
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Other/PivotTableReferenceFiles/PivotSubtotalsSource/output.xlsx
+++ b/ClosedXML.Tests/Resource/Other/PivotTableReferenceFiles/PivotSubtotalsSource/output.xlsx
@@ -514,20 +514,10 @@
       </x:sharedItems>
     </x:cacheField>
     <x:cacheField name="Ship date">
-      <x:sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="1988-05-26T00:00:00" maxDate="1993-10-19T00:00:00" count="4">
-        <x:d v="1988-05-26T00:00:00"/>
-        <x:d v="1988-07-19T00:00:00"/>
-        <x:d v="1988-08-27T00:00:00"/>
-        <x:d v="1993-10-19T00:00:00"/>
-      </x:sharedItems>
+      <x:sharedItems/>
     </x:cacheField>
     <x:cacheField name="Items total">
-      <x:sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="134.85" maxValue="20108" count="4">
-        <x:n v="134.85"/>
-        <x:n v="20108"/>
-        <x:n v="10152"/>
-        <x:n v="1004.8"/>
-      </x:sharedItems>
+      <x:sharedItems/>
     </x:cacheField>
     <x:cacheField name="Tax rate">
       <x:sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="0" count="1">
@@ -535,12 +525,7 @@
       </x:sharedItems>
     </x:cacheField>
     <x:cacheField name="Amount paid">
-      <x:sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="134.85" maxValue="20108" count="4">
-        <x:n v="134.85"/>
-        <x:n v="20108"/>
-        <x:n v="10152"/>
-        <x:n v="1004.8"/>
-      </x:sharedItems>
+      <x:sharedItems/>
     </x:cacheField>
   </x:cacheFields>
   <x:extLst>

</xml_diff>

<commit_message>
Add statistics to pivot cache field.
Field statistics are stored in the file and are available, even if field has no records (save source data = false). Ensure the values are propertly loaded/updated with record values and saved back.

The statistics are not very useful for ClosedXML, but Excel likely uses them for optimized loadings and field structure.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Other/PivotTableReferenceFiles/PivotSubtotalsSource/output.xlsx
+++ b/ClosedXML.Tests/Resource/Other/PivotTableReferenceFiles/PivotSubtotalsSource/output.xlsx
@@ -514,10 +514,10 @@
       </x:sharedItems>
     </x:cacheField>
     <x:cacheField name="Ship date">
-      <x:sharedItems/>
+      <x:sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="1988-05-26T00:00:00" maxDate="1993-10-20T00:00:00"/>
     </x:cacheField>
     <x:cacheField name="Items total">
-      <x:sharedItems/>
+      <x:sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="134.85" maxValue="20108"/>
     </x:cacheField>
     <x:cacheField name="Tax rate">
       <x:sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="0" count="1">
@@ -525,7 +525,7 @@
       </x:sharedItems>
     </x:cacheField>
     <x:cacheField name="Amount paid">
-      <x:sharedItems/>
+      <x:sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="134.85" maxValue="20108"/>
     </x:cacheField>
   </x:cacheFields>
   <x:extLst>

</xml_diff>